<commit_message>
Update trade day data.
</commit_message>
<xml_diff>
--- a/king_index/data/filtered_stocks.xlsx
+++ b/king_index/data/filtered_stocks.xlsx
@@ -1,15 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24026"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\caoxuCarlos.github.io\king_index\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B090D6FD-F645-48B2-AAC2-72A9AC107F3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30060" windowHeight="16032" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -574,8 +591,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -638,6 +655,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -684,7 +709,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -716,9 +741,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -750,6 +793,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -925,11 +986,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I60"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -955,7 +1016,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>11</v>
       </c>
@@ -969,22 +1030,22 @@
         <v>126</v>
       </c>
       <c r="E2">
-        <v>9.2969176995</v>
+        <v>9.2969176994999998</v>
       </c>
       <c r="F2">
-        <v>8.931850969899999</v>
+        <v>8.9318509698999993</v>
       </c>
       <c r="G2">
-        <v>8.4711991898</v>
+        <v>8.4711991898000001</v>
       </c>
       <c r="H2">
-        <v>73.8201</v>
+        <v>73.820099999999996</v>
       </c>
       <c r="I2">
-        <v>99.61239999999999</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
+        <v>99.612399999999994</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>12</v>
       </c>
@@ -998,22 +1059,22 @@
         <v>127</v>
       </c>
       <c r="E3">
-        <v>9.1710109972</v>
+        <v>9.1710109971999998</v>
       </c>
       <c r="F3">
         <v>10.2475007423</v>
       </c>
       <c r="G3">
-        <v>13.3150635194</v>
+        <v>13.315063519400001</v>
       </c>
       <c r="H3">
-        <v>86.7604</v>
+        <v>86.760400000000004</v>
       </c>
       <c r="I3">
-        <v>76.8844</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
+        <v>76.884399999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>30</v>
       </c>
@@ -1027,7 +1088,7 @@
         <v>128</v>
       </c>
       <c r="E4">
-        <v>14.5024128968</v>
+        <v>14.502412896799999</v>
       </c>
       <c r="F4">
         <v>10.1274974289</v>
@@ -1036,13 +1097,13 @@
         <v>16.5202024763</v>
       </c>
       <c r="H4">
-        <v>60.0985</v>
+        <v>60.098500000000001</v>
       </c>
       <c r="I4">
-        <v>274.7619</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
+        <v>274.76190000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>39</v>
       </c>
@@ -1059,19 +1120,19 @@
         <v>17.2762946187</v>
       </c>
       <c r="F5">
-        <v>18.3880787524</v>
+        <v>18.388078752399998</v>
       </c>
       <c r="G5">
-        <v>16.7634821299</v>
+        <v>16.763482129900002</v>
       </c>
       <c r="H5">
-        <v>77.07089999999999</v>
+        <v>77.070899999999995</v>
       </c>
       <c r="I5">
-        <v>75.36450000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+        <v>75.364500000000007</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>40</v>
       </c>
@@ -1085,22 +1146,22 @@
         <v>130</v>
       </c>
       <c r="E6">
-        <v>9.8567396913</v>
+        <v>9.8567396912999996</v>
       </c>
       <c r="F6">
-        <v>15.7071072224</v>
+        <v>15.707107222399999</v>
       </c>
       <c r="G6">
-        <v>13.3895618178</v>
+        <v>13.389561817800001</v>
       </c>
       <c r="H6">
-        <v>66.5483</v>
+        <v>66.548299999999998</v>
       </c>
       <c r="I6">
-        <v>81.068</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
+        <v>81.067999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>50</v>
       </c>
@@ -1114,22 +1175,22 @@
         <v>131</v>
       </c>
       <c r="E7">
-        <v>9.0983924397</v>
+        <v>9.0983924396999996</v>
       </c>
       <c r="F7">
         <v>10.640972847</v>
       </c>
       <c r="G7">
-        <v>12.9930597143</v>
+        <v>12.993059714299999</v>
       </c>
       <c r="H7">
-        <v>55.3975</v>
+        <v>55.397500000000001</v>
       </c>
       <c r="I7">
-        <v>172.2153</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
+        <v>172.21530000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>52</v>
       </c>
@@ -1143,22 +1204,22 @@
         <v>132</v>
       </c>
       <c r="E8">
-        <v>8.515758247599999</v>
+        <v>8.5157582475999991</v>
       </c>
       <c r="F8">
-        <v>9.559501253400001</v>
+        <v>9.5595012534000006</v>
       </c>
       <c r="G8">
         <v>10.8933187031</v>
       </c>
       <c r="H8">
-        <v>47.9388</v>
+        <v>47.938800000000001</v>
       </c>
       <c r="I8">
-        <v>78.2696</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
+        <v>78.269599999999997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>57</v>
       </c>
@@ -1175,19 +1236,19 @@
         <v>12.8364192189</v>
       </c>
       <c r="F9">
-        <v>11.0017237408</v>
+        <v>11.001723740799999</v>
       </c>
       <c r="G9">
         <v>12.1551051382</v>
       </c>
       <c r="H9">
-        <v>70.8411</v>
+        <v>70.841099999999997</v>
       </c>
       <c r="I9">
         <v>168.96</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>62</v>
       </c>
@@ -1201,22 +1262,22 @@
         <v>134</v>
       </c>
       <c r="E10">
-        <v>12.5896184262</v>
+        <v>12.589618426199999</v>
       </c>
       <c r="F10">
-        <v>12.9881046771</v>
+        <v>12.988104677100001</v>
       </c>
       <c r="G10">
-        <v>14.3341875019</v>
+        <v>14.334187501900001</v>
       </c>
       <c r="H10">
-        <v>89.6703</v>
+        <v>89.670299999999997</v>
       </c>
       <c r="I10">
-        <v>38.0087</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
+        <v>38.008699999999997</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>65</v>
       </c>
@@ -1233,19 +1294,19 @@
         <v>10.4986427718</v>
       </c>
       <c r="F11">
-        <v>8.867500554399999</v>
+        <v>8.8675005543999994</v>
       </c>
       <c r="G11">
         <v>10.0158987691</v>
       </c>
       <c r="H11">
-        <v>51.1545</v>
+        <v>51.154499999999999</v>
       </c>
       <c r="I11">
-        <v>45.5782</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9">
+        <v>45.578200000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>72</v>
       </c>
@@ -1259,10 +1320,10 @@
         <v>136</v>
       </c>
       <c r="E12">
-        <v>18.8891279343</v>
+        <v>18.889127934299999</v>
       </c>
       <c r="F12">
-        <v>25.6190411538</v>
+        <v>25.619041153800001</v>
       </c>
       <c r="G12">
         <v>28.379918299</v>
@@ -1271,10 +1332,10 @@
         <v>65.994</v>
       </c>
       <c r="I12">
-        <v>191.2981</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9">
+        <v>191.29810000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>76</v>
       </c>
@@ -1288,22 +1349,22 @@
         <v>137</v>
       </c>
       <c r="E13">
-        <v>19.5248390981</v>
+        <v>19.524839098099999</v>
       </c>
       <c r="F13">
-        <v>21.6929920833</v>
+        <v>21.692992083299998</v>
       </c>
       <c r="G13">
         <v>25.5254067698</v>
       </c>
       <c r="H13">
-        <v>60.9242</v>
+        <v>60.924199999999999</v>
       </c>
       <c r="I13">
         <v>149.7295</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>81</v>
       </c>
@@ -1317,22 +1378,22 @@
         <v>138</v>
       </c>
       <c r="E14">
-        <v>13.8512585265</v>
+        <v>13.851258526500001</v>
       </c>
       <c r="F14">
         <v>11.9794265105</v>
       </c>
       <c r="G14">
-        <v>9.7369340641</v>
+        <v>9.7369340640999997</v>
       </c>
       <c r="H14">
-        <v>52.505</v>
+        <v>52.505000000000003</v>
       </c>
       <c r="I14">
-        <v>40.8805</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
+        <v>40.880499999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>84</v>
       </c>
@@ -1346,22 +1407,22 @@
         <v>139</v>
       </c>
       <c r="E15">
-        <v>9.1322513405</v>
+        <v>9.1322513404999999</v>
       </c>
       <c r="F15">
-        <v>8.624398640600001</v>
+        <v>8.6243986406000008</v>
       </c>
       <c r="G15">
         <v>11.0859262055</v>
       </c>
       <c r="H15">
-        <v>76.735</v>
+        <v>76.734999999999999</v>
       </c>
       <c r="I15">
-        <v>74.1319</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
+        <v>74.131900000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>87</v>
       </c>
@@ -1375,22 +1436,22 @@
         <v>140</v>
       </c>
       <c r="E16">
-        <v>19.2682867685</v>
+        <v>19.268286768500001</v>
       </c>
       <c r="F16">
         <v>22.9140418906</v>
       </c>
       <c r="G16">
-        <v>25.2611707029</v>
+        <v>25.261170702899999</v>
       </c>
       <c r="H16">
-        <v>58.9885</v>
+        <v>58.988500000000002</v>
       </c>
       <c r="I16">
-        <v>186.9104</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+        <v>186.91040000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>89</v>
       </c>
@@ -1407,19 +1468,19 @@
         <v>14.5839798064</v>
       </c>
       <c r="F17">
-        <v>13.5187157768</v>
+        <v>13.518715776800001</v>
       </c>
       <c r="G17">
         <v>11.9208783678</v>
       </c>
       <c r="H17">
-        <v>47.4792</v>
+        <v>47.479199999999999</v>
       </c>
       <c r="I17">
-        <v>71.7466</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+        <v>71.746600000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>90</v>
       </c>
@@ -1433,22 +1494,22 @@
         <v>142</v>
       </c>
       <c r="E18">
-        <v>20.3938054375</v>
+        <v>20.393805437499999</v>
       </c>
       <c r="F18">
-        <v>24.9794297001</v>
+        <v>24.979429700099999</v>
       </c>
       <c r="G18">
         <v>15.2110188849</v>
       </c>
       <c r="H18">
-        <v>56.0363</v>
+        <v>56.036299999999997</v>
       </c>
       <c r="I18">
-        <v>75.9567</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+        <v>75.956699999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>96</v>
       </c>
@@ -1462,7 +1523,7 @@
         <v>143</v>
       </c>
       <c r="E19">
-        <v>11.9071263349</v>
+        <v>11.907126334899999</v>
       </c>
       <c r="F19">
         <v>11.6676518076</v>
@@ -1471,13 +1532,13 @@
         <v>15.3921363759</v>
       </c>
       <c r="H19">
-        <v>54.1298</v>
+        <v>54.129800000000003</v>
       </c>
       <c r="I19">
-        <v>101.3393</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+        <v>101.33929999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>99</v>
       </c>
@@ -1494,19 +1555,19 @@
         <v>22.0006194447</v>
       </c>
       <c r="F20">
-        <v>33.717236709</v>
+        <v>33.717236708999998</v>
       </c>
       <c r="G20">
-        <v>41.6385722166</v>
+        <v>41.638572216599997</v>
       </c>
       <c r="H20">
-        <v>74.61539999999999</v>
+        <v>74.615399999999994</v>
       </c>
       <c r="I20">
         <v>101.1683</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>101</v>
       </c>
@@ -1520,22 +1581,22 @@
         <v>145</v>
       </c>
       <c r="E21">
-        <v>16.085153256</v>
+        <v>16.085153256000002</v>
       </c>
       <c r="F21">
-        <v>14.3800301244</v>
+        <v>14.380030124399999</v>
       </c>
       <c r="G21">
-        <v>16.3056659647</v>
+        <v>16.305665964700001</v>
       </c>
       <c r="H21">
-        <v>68.8687</v>
+        <v>68.868700000000004</v>
       </c>
       <c r="I21">
         <v>108.8164</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>104</v>
       </c>
@@ -1552,19 +1613,19 @@
         <v>10.179910688</v>
       </c>
       <c r="F22">
-        <v>8.7700378755</v>
+        <v>8.7700378754999999</v>
       </c>
       <c r="G22">
-        <v>10.8743505323</v>
+        <v>10.874350532299999</v>
       </c>
       <c r="H22">
-        <v>56.3047</v>
+        <v>56.304699999999997</v>
       </c>
       <c r="I22">
-        <v>91.90900000000001</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
+        <v>91.909000000000006</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>105</v>
       </c>
@@ -1578,22 +1639,22 @@
         <v>147</v>
       </c>
       <c r="E23">
-        <v>12.0557845186</v>
+        <v>12.055784518599999</v>
       </c>
       <c r="F23">
         <v>11.2641319597</v>
       </c>
       <c r="G23">
-        <v>11.3455707408</v>
+        <v>11.345570740799999</v>
       </c>
       <c r="H23">
         <v>55.36</v>
       </c>
       <c r="I23">
-        <v>35.9231</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
+        <v>35.923099999999998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>113</v>
       </c>
@@ -1607,22 +1668,22 @@
         <v>148</v>
       </c>
       <c r="E24">
-        <v>24.9076082185</v>
+        <v>24.907608218499998</v>
       </c>
       <c r="F24">
-        <v>24.2922457437</v>
+        <v>24.292245743700001</v>
       </c>
       <c r="G24">
-        <v>25.6584587898</v>
+        <v>25.658458789800001</v>
       </c>
       <c r="H24">
         <v>47.6235</v>
       </c>
       <c r="I24">
-        <v>55.201</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
+        <v>55.201000000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>121</v>
       </c>
@@ -1636,22 +1697,22 @@
         <v>149</v>
       </c>
       <c r="E25">
-        <v>15.5106992126</v>
+        <v>15.510699212600001</v>
       </c>
       <c r="F25">
-        <v>14.5570209614</v>
+        <v>14.557020961399999</v>
       </c>
       <c r="G25">
-        <v>15.5728336449</v>
+        <v>15.572833644899999</v>
       </c>
       <c r="H25">
-        <v>63.2481</v>
+        <v>63.248100000000001</v>
       </c>
       <c r="I25">
-        <v>77.20820000000001</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
+        <v>77.208200000000005</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>125</v>
       </c>
@@ -1665,22 +1726,22 @@
         <v>150</v>
       </c>
       <c r="E26">
-        <v>12.0557845186</v>
+        <v>12.055784518599999</v>
       </c>
       <c r="F26">
         <v>11.2641319597</v>
       </c>
       <c r="G26">
-        <v>11.3455707408</v>
+        <v>11.345570740799999</v>
       </c>
       <c r="H26">
-        <v>38.2028</v>
+        <v>38.202800000000003</v>
       </c>
       <c r="I26">
         <v>28.3491</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>126</v>
       </c>
@@ -1694,22 +1755,22 @@
         <v>151</v>
       </c>
       <c r="E27">
-        <v>23.8834696295</v>
+        <v>23.883469629499999</v>
       </c>
       <c r="F27">
         <v>27.2421890297</v>
       </c>
       <c r="G27">
-        <v>26.1049503254</v>
+        <v>26.104950325400001</v>
       </c>
       <c r="H27">
-        <v>80.28230000000001</v>
+        <v>80.282300000000006</v>
       </c>
       <c r="I27">
-        <v>105.4463</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9">
+        <v>105.44629999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>128</v>
       </c>
@@ -1726,19 +1787,19 @@
         <v>12.0141644829</v>
       </c>
       <c r="F28">
-        <v>14.3954581415</v>
+        <v>14.395458141500001</v>
       </c>
       <c r="G28">
-        <v>16.6785641034</v>
+        <v>16.678564103399999</v>
       </c>
       <c r="H28">
-        <v>63.9022</v>
+        <v>63.902200000000001</v>
       </c>
       <c r="I28">
-        <v>55.4962</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9">
+        <v>55.496200000000002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>129</v>
       </c>
@@ -1752,22 +1813,22 @@
         <v>153</v>
       </c>
       <c r="E29">
-        <v>23.8772666524</v>
+        <v>23.877266652399999</v>
       </c>
       <c r="F29">
-        <v>21.0593295712</v>
+        <v>21.059329571199999</v>
       </c>
       <c r="G29">
-        <v>19.3397023033</v>
+        <v>19.339702303300001</v>
       </c>
       <c r="H29">
-        <v>58.4352</v>
+        <v>58.435200000000002</v>
       </c>
       <c r="I29">
-        <v>40.7055</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9">
+        <v>40.705500000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>140</v>
       </c>
@@ -1781,7 +1842,7 @@
         <v>154</v>
       </c>
       <c r="E30">
-        <v>13.1539839741</v>
+        <v>13.153983974100001</v>
       </c>
       <c r="F30">
         <v>15.5874389786</v>
@@ -1793,10 +1854,10 @@
         <v>48.1447</v>
       </c>
       <c r="I30">
-        <v>53.3879</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9">
+        <v>53.387900000000002</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>142</v>
       </c>
@@ -1816,16 +1877,16 @@
         <v>24.1124261378</v>
       </c>
       <c r="G31">
-        <v>25.3537482994</v>
+        <v>25.353748299399999</v>
       </c>
       <c r="H31">
-        <v>73.3668</v>
+        <v>73.366799999999998</v>
       </c>
       <c r="I31">
         <v>159.5812</v>
       </c>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>143</v>
       </c>
@@ -1839,22 +1900,22 @@
         <v>156</v>
       </c>
       <c r="E32">
-        <v>16.5593077197</v>
+        <v>16.559307719700001</v>
       </c>
       <c r="F32">
-        <v>18.4157302754</v>
+        <v>18.415730275400001</v>
       </c>
       <c r="G32">
-        <v>20.4820035347</v>
+        <v>20.482003534699999</v>
       </c>
       <c r="H32">
-        <v>53.2689</v>
+        <v>53.268900000000002</v>
       </c>
       <c r="I32">
-        <v>76.89579999999999</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9">
+        <v>76.895799999999994</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>145</v>
       </c>
@@ -1868,22 +1929,22 @@
         <v>157</v>
       </c>
       <c r="E33">
-        <v>23.8525498755</v>
+        <v>23.852549875499999</v>
       </c>
       <c r="F33">
-        <v>25.6974191679</v>
+        <v>25.697419167900001</v>
       </c>
       <c r="G33">
-        <v>21.0476650611</v>
+        <v>21.047665061099998</v>
       </c>
       <c r="H33">
-        <v>59.0609</v>
+        <v>59.060899999999997</v>
       </c>
       <c r="I33">
-        <v>53.7373</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9">
+        <v>53.737299999999998</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>149</v>
       </c>
@@ -1897,22 +1958,22 @@
         <v>158</v>
       </c>
       <c r="E34">
-        <v>8.337117533099999</v>
+        <v>8.3371175330999989</v>
       </c>
       <c r="F34">
         <v>8.0550599877</v>
       </c>
       <c r="G34">
-        <v>9.3535345004</v>
+        <v>9.3535345004000003</v>
       </c>
       <c r="H34">
-        <v>89.6566</v>
+        <v>89.656599999999997</v>
       </c>
       <c r="I34">
-        <v>75.627</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9">
+        <v>75.626999999999995</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>150</v>
       </c>
@@ -1926,22 +1987,22 @@
         <v>159</v>
       </c>
       <c r="E35">
-        <v>32.9541530392</v>
+        <v>32.954153039200001</v>
       </c>
       <c r="F35">
         <v>34.4643499373</v>
       </c>
       <c r="G35">
-        <v>33.1176618919</v>
+        <v>33.117661891899999</v>
       </c>
       <c r="H35">
         <v>42.22</v>
       </c>
       <c r="I35">
-        <v>111.793</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9">
+        <v>111.79300000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>152</v>
       </c>
@@ -1955,7 +2016,7 @@
         <v>160</v>
       </c>
       <c r="E36">
-        <v>14.7495507702</v>
+        <v>14.749550770200001</v>
       </c>
       <c r="F36">
         <v>20.2594663872</v>
@@ -1964,13 +2025,13 @@
         <v>13.6772125099</v>
       </c>
       <c r="H36">
-        <v>69.5942</v>
+        <v>69.594200000000001</v>
       </c>
       <c r="I36">
-        <v>74.5774</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9">
+        <v>74.577399999999997</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>153</v>
       </c>
@@ -1987,19 +2048,19 @@
         <v>12.91865688</v>
       </c>
       <c r="F37">
-        <v>10.9966701392</v>
+        <v>10.996670139200001</v>
       </c>
       <c r="G37">
         <v>10.930546541</v>
       </c>
       <c r="H37">
-        <v>38.3721</v>
+        <v>38.372100000000003</v>
       </c>
       <c r="I37">
-        <v>45.9716</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9">
+        <v>45.971600000000002</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>155</v>
       </c>
@@ -2013,22 +2074,22 @@
         <v>162</v>
       </c>
       <c r="E38">
-        <v>14.727626085</v>
+        <v>14.727626085000001</v>
       </c>
       <c r="F38">
-        <v>15.2419732688</v>
+        <v>15.241973268800001</v>
       </c>
       <c r="G38">
-        <v>25.1170766295</v>
+        <v>25.117076629500001</v>
       </c>
       <c r="H38">
-        <v>45.9459</v>
+        <v>45.945900000000002</v>
       </c>
       <c r="I38">
-        <v>102.3226</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9">
+        <v>102.32259999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>156</v>
       </c>
@@ -2042,22 +2103,22 @@
         <v>163</v>
       </c>
       <c r="E39">
-        <v>17.7938592326</v>
+        <v>17.793859232599999</v>
       </c>
       <c r="F39">
         <v>18.8003531552</v>
       </c>
       <c r="G39">
-        <v>17.4271791719</v>
+        <v>17.427179171900001</v>
       </c>
       <c r="H39">
         <v>46.2376</v>
       </c>
       <c r="I39">
-        <v>67.0857</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9">
+        <v>67.085700000000003</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>157</v>
       </c>
@@ -2077,16 +2138,16 @@
         <v>13.4652012525</v>
       </c>
       <c r="G40">
-        <v>13.9787921097</v>
+        <v>13.978792109700001</v>
       </c>
       <c r="H40">
-        <v>88.607</v>
+        <v>88.606999999999999</v>
       </c>
       <c r="I40">
-        <v>86.333</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9">
+        <v>86.332999999999998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>159</v>
       </c>
@@ -2100,22 +2161,22 @@
         <v>165</v>
       </c>
       <c r="E41">
-        <v>12.1618646851</v>
+        <v>12.161864685099999</v>
       </c>
       <c r="F41">
         <v>12.8082212217</v>
       </c>
       <c r="G41">
-        <v>16.3457620162</v>
+        <v>16.345762016199998</v>
       </c>
       <c r="H41">
-        <v>65.9091</v>
+        <v>65.909099999999995</v>
       </c>
       <c r="I41">
-        <v>91.07980000000001</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9">
+        <v>91.079800000000006</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>160</v>
       </c>
@@ -2129,22 +2190,22 @@
         <v>166</v>
       </c>
       <c r="E42">
-        <v>20.8122532206</v>
+        <v>20.812253220599999</v>
       </c>
       <c r="F42">
-        <v>21.0716121415</v>
+        <v>21.071612141500001</v>
       </c>
       <c r="G42">
-        <v>23.7315277761</v>
+        <v>23.731527776099998</v>
       </c>
       <c r="H42">
-        <v>47.3573</v>
+        <v>47.357300000000002</v>
       </c>
       <c r="I42">
-        <v>34.3284</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9">
+        <v>34.328400000000002</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>162</v>
       </c>
@@ -2164,16 +2225,16 @@
         <v>24.1124261378</v>
       </c>
       <c r="G43">
-        <v>25.3537482994</v>
+        <v>25.353748299399999</v>
       </c>
       <c r="H43">
         <v>47.9846</v>
       </c>
       <c r="I43">
-        <v>90.20820000000001</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9">
+        <v>90.208200000000005</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>164</v>
       </c>
@@ -2187,7 +2248,7 @@
         <v>168</v>
       </c>
       <c r="E44">
-        <v>10.2289830988</v>
+        <v>10.228983098800001</v>
       </c>
       <c r="F44">
         <v>11.5254960192</v>
@@ -2196,13 +2257,13 @@
         <v>12.6939633004</v>
       </c>
       <c r="H44">
-        <v>64.79770000000001</v>
+        <v>64.797700000000006</v>
       </c>
       <c r="I44">
-        <v>124.3885</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9">
+        <v>124.38849999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>165</v>
       </c>
@@ -2216,22 +2277,22 @@
         <v>169</v>
       </c>
       <c r="E45">
-        <v>8.310248182</v>
+        <v>8.3102481820000005</v>
       </c>
       <c r="F45">
         <v>8.316870892899999</v>
       </c>
       <c r="G45">
-        <v>9.3519919404</v>
+        <v>9.3519919403999996</v>
       </c>
       <c r="H45">
-        <v>34.8522</v>
+        <v>34.852200000000003</v>
       </c>
       <c r="I45">
-        <v>63.4899</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9">
+        <v>63.489899999999999</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>167</v>
       </c>
@@ -2248,19 +2309,19 @@
         <v>8.678245197799999</v>
       </c>
       <c r="F46">
-        <v>8.418709659299999</v>
+        <v>8.4187096592999993</v>
       </c>
       <c r="G46">
-        <v>10.4765820043</v>
+        <v>10.476582004300001</v>
       </c>
       <c r="H46">
-        <v>23.1198</v>
+        <v>23.119800000000001</v>
       </c>
       <c r="I46">
-        <v>67.968</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9">
+        <v>67.968000000000004</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>169</v>
       </c>
@@ -2277,19 +2338,19 @@
         <v>18.1410015712</v>
       </c>
       <c r="F47">
-        <v>20.264318745</v>
+        <v>20.264318745000001</v>
       </c>
       <c r="G47">
-        <v>21.9247435173</v>
+        <v>21.924743517300001</v>
       </c>
       <c r="H47">
-        <v>73.7589</v>
+        <v>73.758899999999997</v>
       </c>
       <c r="I47">
         <v>146.9289</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>171</v>
       </c>
@@ -2303,22 +2364,22 @@
         <v>172</v>
       </c>
       <c r="E48">
-        <v>8.9466464317</v>
+        <v>8.9466464316999996</v>
       </c>
       <c r="F48">
-        <v>8.889761805899999</v>
+        <v>8.8897618058999992</v>
       </c>
       <c r="G48">
-        <v>14.7519213202</v>
+        <v>14.751921320199999</v>
       </c>
       <c r="H48">
-        <v>26.789</v>
+        <v>26.789000000000001</v>
       </c>
       <c r="I48">
-        <v>68.12869999999999</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9">
+        <v>68.128699999999995</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>172</v>
       </c>
@@ -2332,22 +2393,22 @@
         <v>173</v>
       </c>
       <c r="E49">
-        <v>29.9744506036</v>
+        <v>29.974450603600001</v>
       </c>
       <c r="F49">
         <v>35.6236512459</v>
       </c>
       <c r="G49">
-        <v>36.9129156891</v>
+        <v>36.912915689099997</v>
       </c>
       <c r="H49">
-        <v>34.6792</v>
+        <v>34.679200000000002</v>
       </c>
       <c r="I49">
-        <v>59.4744</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9">
+        <v>59.474400000000003</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>174</v>
       </c>
@@ -2364,19 +2425,19 @@
         <v>11.0283918293</v>
       </c>
       <c r="F50">
-        <v>8.039359449699999</v>
+        <v>8.0393594496999992</v>
       </c>
       <c r="G50">
-        <v>21.168501548</v>
+        <v>21.168501547999998</v>
       </c>
       <c r="H50">
-        <v>40.6711</v>
+        <v>40.671100000000003</v>
       </c>
       <c r="I50">
-        <v>227.0604</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9">
+        <v>227.06039999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>175</v>
       </c>
@@ -2390,22 +2451,22 @@
         <v>175</v>
       </c>
       <c r="E51">
-        <v>19.9141642357</v>
+        <v>19.914164235699999</v>
       </c>
       <c r="F51">
-        <v>20.2140320342</v>
+        <v>20.214032034199999</v>
       </c>
       <c r="G51">
-        <v>19.5701972225</v>
+        <v>19.570197222499999</v>
       </c>
       <c r="H51">
         <v>40.1282</v>
       </c>
       <c r="I51">
-        <v>65.12730000000001</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9">
+        <v>65.127300000000005</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
         <v>178</v>
       </c>
@@ -2422,19 +2483,19 @@
         <v>12.9228312583</v>
       </c>
       <c r="F52">
-        <v>16.5337592416</v>
+        <v>16.533759241599999</v>
       </c>
       <c r="G52">
-        <v>16.2273985282</v>
+        <v>16.227398528199998</v>
       </c>
       <c r="H52">
-        <v>38.4615</v>
+        <v>38.461500000000001</v>
       </c>
       <c r="I52">
-        <v>51.2195</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9">
+        <v>51.219499999999996</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
         <v>179</v>
       </c>
@@ -2451,19 +2512,19 @@
         <v>21.4058227401</v>
       </c>
       <c r="F53">
-        <v>11.780717982</v>
+        <v>11.780717982000001</v>
       </c>
       <c r="G53">
-        <v>35.0580977729</v>
+        <v>35.058097772899998</v>
       </c>
       <c r="H53">
-        <v>32.9707</v>
+        <v>32.970700000000001</v>
       </c>
       <c r="I53">
-        <v>74.82810000000001</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9">
+        <v>74.828100000000006</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
         <v>182</v>
       </c>
@@ -2477,22 +2538,22 @@
         <v>178</v>
       </c>
       <c r="E54">
-        <v>16.6625022681</v>
+        <v>16.662502268099999</v>
       </c>
       <c r="F54">
         <v>15.8853564317</v>
       </c>
       <c r="G54">
-        <v>15.1427224465</v>
+        <v>15.142722446500001</v>
       </c>
       <c r="H54">
-        <v>49.6183</v>
+        <v>49.618299999999998</v>
       </c>
       <c r="I54">
-        <v>99.2308</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9">
+        <v>99.230800000000002</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <v>183</v>
       </c>
@@ -2506,22 +2567,22 @@
         <v>179</v>
       </c>
       <c r="E55">
-        <v>19.6925917697</v>
+        <v>19.692591769700002</v>
       </c>
       <c r="F55">
-        <v>19.526548807</v>
+        <v>19.526548807000001</v>
       </c>
       <c r="G55">
-        <v>19.0760300615</v>
+        <v>19.076030061499999</v>
       </c>
       <c r="H55">
-        <v>63.9723</v>
+        <v>63.972299999999997</v>
       </c>
       <c r="I55">
-        <v>54.8273</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9">
+        <v>54.827300000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
         <v>185</v>
       </c>
@@ -2535,22 +2596,22 @@
         <v>180</v>
       </c>
       <c r="E56">
-        <v>15.2612085032</v>
+        <v>15.261208503200001</v>
       </c>
       <c r="F56">
-        <v>18.0095701004</v>
+        <v>18.009570100400001</v>
       </c>
       <c r="G56">
-        <v>19.0088856188</v>
+        <v>19.008885618800001</v>
       </c>
       <c r="H56">
-        <v>48.7076</v>
+        <v>48.707599999999999</v>
       </c>
       <c r="I56">
-        <v>72.9464</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9">
+        <v>72.946399999999997</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>186</v>
       </c>
@@ -2567,19 +2628,19 @@
         <v>10.6191178046</v>
       </c>
       <c r="F57">
-        <v>13.5482601264</v>
+        <v>13.548260126400001</v>
       </c>
       <c r="G57">
-        <v>17.2918903103</v>
+        <v>17.291890310300001</v>
       </c>
       <c r="H57">
-        <v>43.7619</v>
+        <v>43.761899999999997</v>
       </c>
       <c r="I57">
-        <v>96.84869999999999</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9">
+        <v>96.848699999999994</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
         <v>188</v>
       </c>
@@ -2593,22 +2654,22 @@
         <v>182</v>
       </c>
       <c r="E58">
-        <v>23.7035077268</v>
+        <v>23.703507726800002</v>
       </c>
       <c r="F58">
-        <v>30.0837133869</v>
+        <v>30.083713386900001</v>
       </c>
       <c r="G58">
-        <v>22.6542502992</v>
+        <v>22.654250299200001</v>
       </c>
       <c r="H58">
-        <v>83.542</v>
+        <v>83.542000000000002</v>
       </c>
       <c r="I58">
-        <v>53.4259</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9">
+        <v>53.425899999999999</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
         <v>189</v>
       </c>
@@ -2622,22 +2683,22 @@
         <v>183</v>
       </c>
       <c r="E59">
-        <v>32.4474587604</v>
+        <v>32.447458760400004</v>
       </c>
       <c r="F59">
-        <v>34.0622182315</v>
+        <v>34.062218231499998</v>
       </c>
       <c r="G59">
         <v>35.1523113298</v>
       </c>
       <c r="H59">
-        <v>67.23050000000001</v>
+        <v>67.230500000000006</v>
       </c>
       <c r="I59">
-        <v>76.64239999999999</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9">
+        <v>76.642399999999995</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
         <v>194</v>
       </c>
@@ -2654,16 +2715,16 @@
         <v>27.5285049035</v>
       </c>
       <c r="F60">
-        <v>34.9968967693</v>
+        <v>34.996896769300001</v>
       </c>
       <c r="G60">
-        <v>51.2477477438</v>
+        <v>51.247747743799998</v>
       </c>
       <c r="H60">
         <v>71.9559</v>
       </c>
       <c r="I60">
-        <v>99.8698</v>
+        <v>99.869799999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>